<commit_message>
bo sung data - test tinh luong thieu ngay
</commit_message>
<xml_diff>
--- a/import.xlsx
+++ b/import.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1\Desktop\HTTTDN\ManageLegoShop_DesktopApp_V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1804F4-50AF-4192-AB20-E31788CC6B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637708F3-1D14-45B2-93B4-F35593490A1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11865" yWindow="1710" windowWidth="14250" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
   <si>
     <t>Mã NV (Số/Chữ)</t>
   </si>
@@ -45,6 +45,12 @@
   </si>
   <si>
     <t>Giờ Ra (MM-dd-yyyy HH:mm)</t>
+  </si>
+  <si>
+    <t>11/31/2025  8:00:00 AM</t>
+  </si>
+  <si>
+    <t>11/31/2025  5:00:00 PM</t>
   </si>
 </sst>
 </file>
@@ -429,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C404"/>
+  <dimension ref="A1:C683"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
@@ -4881,6 +4887,3075 @@
         <v>46053.708333333336</v>
       </c>
     </row>
+    <row r="405" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A405" s="2">
+        <v>1</v>
+      </c>
+      <c r="B405" s="3">
+        <v>45992.333333333336</v>
+      </c>
+      <c r="C405" s="3">
+        <v>45992.708333333336</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A406" s="2">
+        <v>1</v>
+      </c>
+      <c r="B406" s="3">
+        <v>45993.333333333336</v>
+      </c>
+      <c r="C406" s="3">
+        <v>45993.708333333336</v>
+      </c>
+    </row>
+    <row r="407" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A407" s="2">
+        <v>1</v>
+      </c>
+      <c r="B407" s="3">
+        <v>45994.333333333336</v>
+      </c>
+      <c r="C407" s="3">
+        <v>45994.708333333336</v>
+      </c>
+    </row>
+    <row r="408" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A408" s="2">
+        <v>1</v>
+      </c>
+      <c r="B408" s="3">
+        <v>45995.333333333336</v>
+      </c>
+      <c r="C408" s="3">
+        <v>45995.708333333336</v>
+      </c>
+    </row>
+    <row r="409" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A409" s="2">
+        <v>1</v>
+      </c>
+      <c r="B409" s="3">
+        <v>45996.333333333336</v>
+      </c>
+      <c r="C409" s="3">
+        <v>45996.708333333336</v>
+      </c>
+    </row>
+    <row r="410" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A410" s="2">
+        <v>1</v>
+      </c>
+      <c r="B410" s="3">
+        <v>45997.333333333336</v>
+      </c>
+      <c r="C410" s="3">
+        <v>45997.708333333336</v>
+      </c>
+    </row>
+    <row r="411" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A411" s="2">
+        <v>1</v>
+      </c>
+      <c r="B411" s="3">
+        <v>45998.333333333336</v>
+      </c>
+      <c r="C411" s="3">
+        <v>45998.708333333336</v>
+      </c>
+    </row>
+    <row r="412" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A412" s="2">
+        <v>1</v>
+      </c>
+      <c r="B412" s="3">
+        <v>45999.333333333336</v>
+      </c>
+      <c r="C412" s="3">
+        <v>45999.708333333336</v>
+      </c>
+    </row>
+    <row r="413" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A413" s="2">
+        <v>1</v>
+      </c>
+      <c r="B413" s="3">
+        <v>46000.333333333336</v>
+      </c>
+      <c r="C413" s="3">
+        <v>46000.708333333336</v>
+      </c>
+    </row>
+    <row r="414" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A414" s="2">
+        <v>1</v>
+      </c>
+      <c r="B414" s="3">
+        <v>46001.333333333336</v>
+      </c>
+      <c r="C414" s="3">
+        <v>46001.708333333336</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A415" s="2">
+        <v>1</v>
+      </c>
+      <c r="B415" s="3">
+        <v>46002.333333333336</v>
+      </c>
+      <c r="C415" s="3">
+        <v>46002.708333333336</v>
+      </c>
+    </row>
+    <row r="416" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A416" s="2">
+        <v>1</v>
+      </c>
+      <c r="B416" s="3">
+        <v>46003.333333333336</v>
+      </c>
+      <c r="C416" s="3">
+        <v>46003.708333333336</v>
+      </c>
+    </row>
+    <row r="417" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A417" s="2">
+        <v>1</v>
+      </c>
+      <c r="B417" s="3">
+        <v>46004.333333333336</v>
+      </c>
+      <c r="C417" s="3">
+        <v>46004.708333333336</v>
+      </c>
+    </row>
+    <row r="418" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A418" s="2">
+        <v>1</v>
+      </c>
+      <c r="B418" s="3">
+        <v>46005.333333333336</v>
+      </c>
+      <c r="C418" s="3">
+        <v>46005.708333333336</v>
+      </c>
+    </row>
+    <row r="419" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A419" s="2">
+        <v>1</v>
+      </c>
+      <c r="B419" s="3">
+        <v>46006.333333333336</v>
+      </c>
+      <c r="C419" s="3">
+        <v>46006.708333333336</v>
+      </c>
+    </row>
+    <row r="420" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A420" s="2">
+        <v>1</v>
+      </c>
+      <c r="B420" s="3">
+        <v>46007.333333333336</v>
+      </c>
+      <c r="C420" s="3">
+        <v>46007.708333333336</v>
+      </c>
+    </row>
+    <row r="421" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A421" s="2">
+        <v>1</v>
+      </c>
+      <c r="B421" s="3">
+        <v>46008.333333333336</v>
+      </c>
+      <c r="C421" s="3">
+        <v>46008.708333333336</v>
+      </c>
+    </row>
+    <row r="422" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A422" s="2">
+        <v>1</v>
+      </c>
+      <c r="B422" s="3">
+        <v>46009.333333333336</v>
+      </c>
+      <c r="C422" s="3">
+        <v>46009.708333333336</v>
+      </c>
+    </row>
+    <row r="423" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A423" s="2">
+        <v>1</v>
+      </c>
+      <c r="B423" s="3">
+        <v>46010.333333333336</v>
+      </c>
+      <c r="C423" s="3">
+        <v>46010.708333333336</v>
+      </c>
+    </row>
+    <row r="424" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A424" s="2">
+        <v>1</v>
+      </c>
+      <c r="B424" s="3">
+        <v>46011.333333333336</v>
+      </c>
+      <c r="C424" s="3">
+        <v>46011.708333333336</v>
+      </c>
+    </row>
+    <row r="425" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A425" s="2">
+        <v>1</v>
+      </c>
+      <c r="B425" s="3">
+        <v>46012.333333333336</v>
+      </c>
+      <c r="C425" s="3">
+        <v>46012.708333333336</v>
+      </c>
+    </row>
+    <row r="426" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A426" s="2">
+        <v>1</v>
+      </c>
+      <c r="B426" s="3">
+        <v>46013.333333333336</v>
+      </c>
+      <c r="C426" s="3">
+        <v>46013.708333333336</v>
+      </c>
+    </row>
+    <row r="427" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A427" s="2">
+        <v>1</v>
+      </c>
+      <c r="B427" s="3">
+        <v>46014.333333333336</v>
+      </c>
+      <c r="C427" s="3">
+        <v>46014.708333333336</v>
+      </c>
+    </row>
+    <row r="428" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A428" s="2">
+        <v>1</v>
+      </c>
+      <c r="B428" s="3">
+        <v>46015.333333333336</v>
+      </c>
+      <c r="C428" s="3">
+        <v>46015.708333333336</v>
+      </c>
+    </row>
+    <row r="429" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A429" s="2">
+        <v>1</v>
+      </c>
+      <c r="B429" s="3">
+        <v>46016.333333333336</v>
+      </c>
+      <c r="C429" s="3">
+        <v>46016.708333333336</v>
+      </c>
+    </row>
+    <row r="430" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A430" s="2">
+        <v>1</v>
+      </c>
+      <c r="B430" s="3">
+        <v>46017.333333333336</v>
+      </c>
+      <c r="C430" s="3">
+        <v>46017.708333333336</v>
+      </c>
+    </row>
+    <row r="431" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A431" s="2">
+        <v>1</v>
+      </c>
+      <c r="B431" s="3">
+        <v>46018.333333333336</v>
+      </c>
+      <c r="C431" s="3">
+        <v>46018.708333333336</v>
+      </c>
+    </row>
+    <row r="432" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A432" s="2">
+        <v>1</v>
+      </c>
+      <c r="B432" s="3">
+        <v>46019.333333333336</v>
+      </c>
+      <c r="C432" s="3">
+        <v>46019.708333333336</v>
+      </c>
+    </row>
+    <row r="433" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A433" s="2">
+        <v>1</v>
+      </c>
+      <c r="B433" s="3">
+        <v>46020.333333333336</v>
+      </c>
+      <c r="C433" s="3">
+        <v>46020.708333333336</v>
+      </c>
+    </row>
+    <row r="434" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A434" s="2">
+        <v>1</v>
+      </c>
+      <c r="B434" s="3">
+        <v>46021.333333333336</v>
+      </c>
+      <c r="C434" s="3">
+        <v>46021.708333333336</v>
+      </c>
+    </row>
+    <row r="435" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A435" s="2">
+        <v>1</v>
+      </c>
+      <c r="B435" s="3">
+        <v>46022.333333333336</v>
+      </c>
+      <c r="C435" s="3">
+        <v>46022.708333333336</v>
+      </c>
+    </row>
+    <row r="436" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A436" s="2">
+        <v>2</v>
+      </c>
+      <c r="B436" s="3">
+        <v>45992.333333333336</v>
+      </c>
+      <c r="C436" s="3">
+        <v>45992.708333333336</v>
+      </c>
+    </row>
+    <row r="437" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A437" s="2">
+        <v>2</v>
+      </c>
+      <c r="B437" s="3">
+        <v>45993.333333333336</v>
+      </c>
+      <c r="C437" s="3">
+        <v>45993.708333333336</v>
+      </c>
+    </row>
+    <row r="438" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A438" s="2">
+        <v>2</v>
+      </c>
+      <c r="B438" s="3">
+        <v>45994.333333333336</v>
+      </c>
+      <c r="C438" s="3">
+        <v>45994.708333333336</v>
+      </c>
+    </row>
+    <row r="439" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A439" s="2">
+        <v>2</v>
+      </c>
+      <c r="B439" s="3">
+        <v>45995.333333333336</v>
+      </c>
+      <c r="C439" s="3">
+        <v>45995.708333333336</v>
+      </c>
+    </row>
+    <row r="440" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A440" s="2">
+        <v>2</v>
+      </c>
+      <c r="B440" s="3">
+        <v>45996.333333333336</v>
+      </c>
+      <c r="C440" s="3">
+        <v>45996.708333333336</v>
+      </c>
+    </row>
+    <row r="441" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A441" s="2">
+        <v>2</v>
+      </c>
+      <c r="B441" s="3">
+        <v>45997.333333333336</v>
+      </c>
+      <c r="C441" s="3">
+        <v>45997.708333333336</v>
+      </c>
+    </row>
+    <row r="442" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A442" s="2">
+        <v>2</v>
+      </c>
+      <c r="B442" s="3">
+        <v>45998.333333333336</v>
+      </c>
+      <c r="C442" s="3">
+        <v>45998.708333333336</v>
+      </c>
+    </row>
+    <row r="443" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A443" s="2">
+        <v>2</v>
+      </c>
+      <c r="B443" s="3">
+        <v>45999.333333333336</v>
+      </c>
+      <c r="C443" s="3">
+        <v>45999.708333333336</v>
+      </c>
+    </row>
+    <row r="444" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A444" s="2">
+        <v>2</v>
+      </c>
+      <c r="B444" s="3">
+        <v>46000.333333333336</v>
+      </c>
+      <c r="C444" s="3">
+        <v>46000.708333333336</v>
+      </c>
+    </row>
+    <row r="445" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A445" s="2">
+        <v>2</v>
+      </c>
+      <c r="B445" s="3">
+        <v>46001.333333333336</v>
+      </c>
+      <c r="C445" s="3">
+        <v>46001.708333333336</v>
+      </c>
+    </row>
+    <row r="446" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A446" s="2">
+        <v>2</v>
+      </c>
+      <c r="B446" s="3">
+        <v>46002.333333333336</v>
+      </c>
+      <c r="C446" s="3">
+        <v>46002.708333333336</v>
+      </c>
+    </row>
+    <row r="447" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A447" s="2">
+        <v>2</v>
+      </c>
+      <c r="B447" s="3">
+        <v>46003.333333333336</v>
+      </c>
+      <c r="C447" s="3">
+        <v>46003.708333333336</v>
+      </c>
+    </row>
+    <row r="448" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A448" s="2">
+        <v>2</v>
+      </c>
+      <c r="B448" s="3">
+        <v>46004.333333333336</v>
+      </c>
+      <c r="C448" s="3">
+        <v>46004.708333333336</v>
+      </c>
+    </row>
+    <row r="449" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A449" s="2">
+        <v>2</v>
+      </c>
+      <c r="B449" s="3">
+        <v>46005.333333333336</v>
+      </c>
+      <c r="C449" s="3">
+        <v>46005.708333333336</v>
+      </c>
+    </row>
+    <row r="450" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A450" s="2">
+        <v>2</v>
+      </c>
+      <c r="B450" s="3">
+        <v>46006.333333333336</v>
+      </c>
+      <c r="C450" s="3">
+        <v>46006.708333333336</v>
+      </c>
+    </row>
+    <row r="451" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A451" s="2">
+        <v>2</v>
+      </c>
+      <c r="B451" s="3">
+        <v>46007.333333333336</v>
+      </c>
+      <c r="C451" s="3">
+        <v>46007.708333333336</v>
+      </c>
+    </row>
+    <row r="452" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A452" s="2">
+        <v>2</v>
+      </c>
+      <c r="B452" s="3">
+        <v>46008.333333333336</v>
+      </c>
+      <c r="C452" s="3">
+        <v>46008.708333333336</v>
+      </c>
+    </row>
+    <row r="453" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A453" s="2">
+        <v>2</v>
+      </c>
+      <c r="B453" s="3">
+        <v>46009.333333333336</v>
+      </c>
+      <c r="C453" s="3">
+        <v>46009.708333333336</v>
+      </c>
+    </row>
+    <row r="454" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A454" s="2">
+        <v>2</v>
+      </c>
+      <c r="B454" s="3">
+        <v>46010.333333333336</v>
+      </c>
+      <c r="C454" s="3">
+        <v>46010.708333333336</v>
+      </c>
+    </row>
+    <row r="455" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A455" s="2">
+        <v>2</v>
+      </c>
+      <c r="B455" s="3">
+        <v>46011.333333333336</v>
+      </c>
+      <c r="C455" s="3">
+        <v>46011.708333333336</v>
+      </c>
+    </row>
+    <row r="456" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A456" s="2">
+        <v>2</v>
+      </c>
+      <c r="B456" s="3">
+        <v>46012.333333333336</v>
+      </c>
+      <c r="C456" s="3">
+        <v>46012.708333333336</v>
+      </c>
+    </row>
+    <row r="457" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A457" s="2">
+        <v>2</v>
+      </c>
+      <c r="B457" s="3">
+        <v>46013.333333333336</v>
+      </c>
+      <c r="C457" s="3">
+        <v>46013.708333333336</v>
+      </c>
+    </row>
+    <row r="458" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A458" s="2">
+        <v>2</v>
+      </c>
+      <c r="B458" s="3">
+        <v>46014.333333333336</v>
+      </c>
+      <c r="C458" s="3">
+        <v>46014.708333333336</v>
+      </c>
+    </row>
+    <row r="459" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A459" s="2">
+        <v>2</v>
+      </c>
+      <c r="B459" s="3">
+        <v>46015.333333333336</v>
+      </c>
+      <c r="C459" s="3">
+        <v>46015.708333333336</v>
+      </c>
+    </row>
+    <row r="460" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A460" s="2">
+        <v>2</v>
+      </c>
+      <c r="B460" s="3">
+        <v>46016.333333333336</v>
+      </c>
+      <c r="C460" s="3">
+        <v>46016.708333333336</v>
+      </c>
+    </row>
+    <row r="461" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A461" s="2">
+        <v>2</v>
+      </c>
+      <c r="B461" s="3">
+        <v>46017.333333333336</v>
+      </c>
+      <c r="C461" s="3">
+        <v>46017.708333333336</v>
+      </c>
+    </row>
+    <row r="462" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A462" s="2">
+        <v>2</v>
+      </c>
+      <c r="B462" s="3">
+        <v>46018.333333333336</v>
+      </c>
+      <c r="C462" s="3">
+        <v>46018.708333333336</v>
+      </c>
+    </row>
+    <row r="463" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A463" s="2">
+        <v>2</v>
+      </c>
+      <c r="B463" s="3">
+        <v>46019.333333333336</v>
+      </c>
+      <c r="C463" s="3">
+        <v>46019.708333333336</v>
+      </c>
+    </row>
+    <row r="464" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A464" s="2">
+        <v>2</v>
+      </c>
+      <c r="B464" s="3">
+        <v>46020.333333333336</v>
+      </c>
+      <c r="C464" s="3">
+        <v>46020.708333333336</v>
+      </c>
+    </row>
+    <row r="465" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A465" s="2">
+        <v>2</v>
+      </c>
+      <c r="B465" s="3">
+        <v>46021.333333333336</v>
+      </c>
+      <c r="C465" s="3">
+        <v>46021.708333333336</v>
+      </c>
+    </row>
+    <row r="466" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A466" s="2">
+        <v>2</v>
+      </c>
+      <c r="B466" s="3">
+        <v>46022.333333333336</v>
+      </c>
+      <c r="C466" s="3">
+        <v>46022.708333333336</v>
+      </c>
+    </row>
+    <row r="467" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A467" s="2">
+        <v>3</v>
+      </c>
+      <c r="B467" s="3">
+        <v>45992.333333333336</v>
+      </c>
+      <c r="C467" s="3">
+        <v>45992.708333333336</v>
+      </c>
+    </row>
+    <row r="468" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A468" s="2">
+        <v>3</v>
+      </c>
+      <c r="B468" s="3">
+        <v>45993.333333333336</v>
+      </c>
+      <c r="C468" s="3">
+        <v>45993.708333333336</v>
+      </c>
+    </row>
+    <row r="469" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A469" s="2">
+        <v>3</v>
+      </c>
+      <c r="B469" s="3">
+        <v>45994.333333333336</v>
+      </c>
+      <c r="C469" s="3">
+        <v>45994.708333333336</v>
+      </c>
+    </row>
+    <row r="470" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A470" s="2">
+        <v>3</v>
+      </c>
+      <c r="B470" s="3">
+        <v>45995.333333333336</v>
+      </c>
+      <c r="C470" s="3">
+        <v>45995.708333333336</v>
+      </c>
+    </row>
+    <row r="471" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A471" s="2">
+        <v>3</v>
+      </c>
+      <c r="B471" s="3">
+        <v>45996.333333333336</v>
+      </c>
+      <c r="C471" s="3">
+        <v>45996.708333333336</v>
+      </c>
+    </row>
+    <row r="472" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A472" s="2">
+        <v>3</v>
+      </c>
+      <c r="B472" s="3">
+        <v>45997.333333333336</v>
+      </c>
+      <c r="C472" s="3">
+        <v>45997.708333333336</v>
+      </c>
+    </row>
+    <row r="473" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A473" s="2">
+        <v>3</v>
+      </c>
+      <c r="B473" s="3">
+        <v>45998.333333333336</v>
+      </c>
+      <c r="C473" s="3">
+        <v>45998.708333333336</v>
+      </c>
+    </row>
+    <row r="474" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A474" s="2">
+        <v>3</v>
+      </c>
+      <c r="B474" s="3">
+        <v>45999.333333333336</v>
+      </c>
+      <c r="C474" s="3">
+        <v>45999.708333333336</v>
+      </c>
+    </row>
+    <row r="475" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A475" s="2">
+        <v>3</v>
+      </c>
+      <c r="B475" s="3">
+        <v>46000.333333333336</v>
+      </c>
+      <c r="C475" s="3">
+        <v>46000.708333333336</v>
+      </c>
+    </row>
+    <row r="476" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A476" s="2">
+        <v>3</v>
+      </c>
+      <c r="B476" s="3">
+        <v>46001.333333333336</v>
+      </c>
+      <c r="C476" s="3">
+        <v>46001.708333333336</v>
+      </c>
+    </row>
+    <row r="477" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A477" s="2">
+        <v>3</v>
+      </c>
+      <c r="B477" s="3">
+        <v>46002.333333333336</v>
+      </c>
+      <c r="C477" s="3">
+        <v>46002.708333333336</v>
+      </c>
+    </row>
+    <row r="478" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A478" s="2">
+        <v>3</v>
+      </c>
+      <c r="B478" s="3">
+        <v>46003.333333333336</v>
+      </c>
+      <c r="C478" s="3">
+        <v>46003.708333333336</v>
+      </c>
+    </row>
+    <row r="479" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A479" s="2">
+        <v>3</v>
+      </c>
+      <c r="B479" s="3">
+        <v>46004.333333333336</v>
+      </c>
+      <c r="C479" s="3">
+        <v>46004.708333333336</v>
+      </c>
+    </row>
+    <row r="480" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A480" s="2">
+        <v>3</v>
+      </c>
+      <c r="B480" s="3">
+        <v>46005.333333333336</v>
+      </c>
+      <c r="C480" s="3">
+        <v>46005.708333333336</v>
+      </c>
+    </row>
+    <row r="481" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A481" s="2">
+        <v>3</v>
+      </c>
+      <c r="B481" s="3">
+        <v>46006.333333333336</v>
+      </c>
+      <c r="C481" s="3">
+        <v>46006.708333333336</v>
+      </c>
+    </row>
+    <row r="482" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A482" s="2">
+        <v>3</v>
+      </c>
+      <c r="B482" s="3">
+        <v>46007.333333333336</v>
+      </c>
+      <c r="C482" s="3">
+        <v>46007.708333333336</v>
+      </c>
+    </row>
+    <row r="483" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A483" s="2">
+        <v>3</v>
+      </c>
+      <c r="B483" s="3">
+        <v>46008.333333333336</v>
+      </c>
+      <c r="C483" s="3">
+        <v>46008.708333333336</v>
+      </c>
+    </row>
+    <row r="484" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A484" s="2">
+        <v>3</v>
+      </c>
+      <c r="B484" s="3">
+        <v>46009.333333333336</v>
+      </c>
+      <c r="C484" s="3">
+        <v>46009.708333333336</v>
+      </c>
+    </row>
+    <row r="485" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A485" s="2">
+        <v>3</v>
+      </c>
+      <c r="B485" s="3">
+        <v>46010.333333333336</v>
+      </c>
+      <c r="C485" s="3">
+        <v>46010.708333333336</v>
+      </c>
+    </row>
+    <row r="486" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A486" s="2">
+        <v>3</v>
+      </c>
+      <c r="B486" s="3">
+        <v>46011.333333333336</v>
+      </c>
+      <c r="C486" s="3">
+        <v>46011.708333333336</v>
+      </c>
+    </row>
+    <row r="487" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A487" s="2">
+        <v>3</v>
+      </c>
+      <c r="B487" s="3">
+        <v>46012.333333333336</v>
+      </c>
+      <c r="C487" s="3">
+        <v>46012.708333333336</v>
+      </c>
+    </row>
+    <row r="488" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A488" s="2">
+        <v>3</v>
+      </c>
+      <c r="B488" s="3">
+        <v>46013.333333333336</v>
+      </c>
+      <c r="C488" s="3">
+        <v>46013.708333333336</v>
+      </c>
+    </row>
+    <row r="489" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A489" s="2">
+        <v>3</v>
+      </c>
+      <c r="B489" s="3">
+        <v>46014.333333333336</v>
+      </c>
+      <c r="C489" s="3">
+        <v>46014.708333333336</v>
+      </c>
+    </row>
+    <row r="490" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A490" s="2">
+        <v>3</v>
+      </c>
+      <c r="B490" s="3">
+        <v>46015.333333333336</v>
+      </c>
+      <c r="C490" s="3">
+        <v>46015.708333333336</v>
+      </c>
+    </row>
+    <row r="491" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A491" s="2">
+        <v>3</v>
+      </c>
+      <c r="B491" s="3">
+        <v>46016.333333333336</v>
+      </c>
+      <c r="C491" s="3">
+        <v>46016.708333333336</v>
+      </c>
+    </row>
+    <row r="492" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A492" s="2">
+        <v>3</v>
+      </c>
+      <c r="B492" s="3">
+        <v>46017.333333333336</v>
+      </c>
+      <c r="C492" s="3">
+        <v>46017.708333333336</v>
+      </c>
+    </row>
+    <row r="493" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A493" s="2">
+        <v>3</v>
+      </c>
+      <c r="B493" s="3">
+        <v>46018.333333333336</v>
+      </c>
+      <c r="C493" s="3">
+        <v>46018.708333333336</v>
+      </c>
+    </row>
+    <row r="494" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A494" s="2">
+        <v>3</v>
+      </c>
+      <c r="B494" s="3">
+        <v>46019.333333333336</v>
+      </c>
+      <c r="C494" s="3">
+        <v>46019.708333333336</v>
+      </c>
+    </row>
+    <row r="495" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A495" s="2">
+        <v>3</v>
+      </c>
+      <c r="B495" s="3">
+        <v>46020.333333333336</v>
+      </c>
+      <c r="C495" s="3">
+        <v>46020.708333333336</v>
+      </c>
+    </row>
+    <row r="496" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A496" s="2">
+        <v>3</v>
+      </c>
+      <c r="B496" s="3">
+        <v>46021.333333333336</v>
+      </c>
+      <c r="C496" s="3">
+        <v>46021.708333333336</v>
+      </c>
+    </row>
+    <row r="497" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A497" s="2">
+        <v>3</v>
+      </c>
+      <c r="B497" s="3">
+        <v>46022.333333333336</v>
+      </c>
+      <c r="C497" s="3">
+        <v>46022.708333333336</v>
+      </c>
+    </row>
+    <row r="498" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A498" s="2">
+        <v>1</v>
+      </c>
+      <c r="B498" s="3">
+        <v>45962.333333333336</v>
+      </c>
+      <c r="C498" s="3">
+        <v>45962.708333333336</v>
+      </c>
+    </row>
+    <row r="499" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A499" s="2">
+        <v>1</v>
+      </c>
+      <c r="B499" s="3">
+        <v>45963.333333333336</v>
+      </c>
+      <c r="C499" s="3">
+        <v>45963.708333333336</v>
+      </c>
+    </row>
+    <row r="500" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A500" s="2">
+        <v>1</v>
+      </c>
+      <c r="B500" s="3">
+        <v>45964.333333333336</v>
+      </c>
+      <c r="C500" s="3">
+        <v>45964.708333333336</v>
+      </c>
+    </row>
+    <row r="501" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A501" s="2">
+        <v>1</v>
+      </c>
+      <c r="B501" s="3">
+        <v>45965.333333333336</v>
+      </c>
+      <c r="C501" s="3">
+        <v>45965.708333333336</v>
+      </c>
+    </row>
+    <row r="502" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A502" s="2">
+        <v>1</v>
+      </c>
+      <c r="B502" s="3">
+        <v>45966.333333333336</v>
+      </c>
+      <c r="C502" s="3">
+        <v>45966.708333333336</v>
+      </c>
+    </row>
+    <row r="503" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A503" s="2">
+        <v>1</v>
+      </c>
+      <c r="B503" s="3">
+        <v>45967.333333333336</v>
+      </c>
+      <c r="C503" s="3">
+        <v>45967.708333333336</v>
+      </c>
+    </row>
+    <row r="504" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A504" s="2">
+        <v>1</v>
+      </c>
+      <c r="B504" s="3">
+        <v>45968.333333333336</v>
+      </c>
+      <c r="C504" s="3">
+        <v>45968.708333333336</v>
+      </c>
+    </row>
+    <row r="505" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A505" s="2">
+        <v>1</v>
+      </c>
+      <c r="B505" s="3">
+        <v>45969.333333333336</v>
+      </c>
+      <c r="C505" s="3">
+        <v>45969.708333333336</v>
+      </c>
+    </row>
+    <row r="506" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A506" s="2">
+        <v>1</v>
+      </c>
+      <c r="B506" s="3">
+        <v>45970.333333333336</v>
+      </c>
+      <c r="C506" s="3">
+        <v>45970.708333333336</v>
+      </c>
+    </row>
+    <row r="507" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A507" s="2">
+        <v>1</v>
+      </c>
+      <c r="B507" s="3">
+        <v>45971.333333333336</v>
+      </c>
+      <c r="C507" s="3">
+        <v>45971.708333333336</v>
+      </c>
+    </row>
+    <row r="508" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A508" s="2">
+        <v>1</v>
+      </c>
+      <c r="B508" s="3">
+        <v>45972.333333333336</v>
+      </c>
+      <c r="C508" s="3">
+        <v>45972.708333333336</v>
+      </c>
+    </row>
+    <row r="509" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A509" s="2">
+        <v>1</v>
+      </c>
+      <c r="B509" s="3">
+        <v>45973.333333333336</v>
+      </c>
+      <c r="C509" s="3">
+        <v>45973.708333333336</v>
+      </c>
+    </row>
+    <row r="510" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A510" s="2">
+        <v>1</v>
+      </c>
+      <c r="B510" s="3">
+        <v>45974.333333333336</v>
+      </c>
+      <c r="C510" s="3">
+        <v>45974.708333333336</v>
+      </c>
+    </row>
+    <row r="511" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A511" s="2">
+        <v>1</v>
+      </c>
+      <c r="B511" s="3">
+        <v>45975.333333333336</v>
+      </c>
+      <c r="C511" s="3">
+        <v>45975.708333333336</v>
+      </c>
+    </row>
+    <row r="512" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A512" s="2">
+        <v>1</v>
+      </c>
+      <c r="B512" s="3">
+        <v>45976.333333333336</v>
+      </c>
+      <c r="C512" s="3">
+        <v>45976.708333333336</v>
+      </c>
+    </row>
+    <row r="513" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A513" s="2">
+        <v>1</v>
+      </c>
+      <c r="B513" s="3">
+        <v>45977.333333333336</v>
+      </c>
+      <c r="C513" s="3">
+        <v>45977.708333333336</v>
+      </c>
+    </row>
+    <row r="514" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A514" s="2">
+        <v>1</v>
+      </c>
+      <c r="B514" s="3">
+        <v>45978.333333333336</v>
+      </c>
+      <c r="C514" s="3">
+        <v>45978.708333333336</v>
+      </c>
+    </row>
+    <row r="515" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A515" s="2">
+        <v>1</v>
+      </c>
+      <c r="B515" s="3">
+        <v>45979.333333333336</v>
+      </c>
+      <c r="C515" s="3">
+        <v>45979.708333333336</v>
+      </c>
+    </row>
+    <row r="516" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A516" s="2">
+        <v>1</v>
+      </c>
+      <c r="B516" s="3">
+        <v>45980.333333333336</v>
+      </c>
+      <c r="C516" s="3">
+        <v>45980.708333333336</v>
+      </c>
+    </row>
+    <row r="517" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A517" s="2">
+        <v>1</v>
+      </c>
+      <c r="B517" s="3">
+        <v>45981.333333333336</v>
+      </c>
+      <c r="C517" s="3">
+        <v>45981.708333333336</v>
+      </c>
+    </row>
+    <row r="518" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A518" s="2">
+        <v>1</v>
+      </c>
+      <c r="B518" s="3">
+        <v>45982.333333333336</v>
+      </c>
+      <c r="C518" s="3">
+        <v>45982.708333333336</v>
+      </c>
+    </row>
+    <row r="519" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A519" s="2">
+        <v>1</v>
+      </c>
+      <c r="B519" s="3">
+        <v>45983.333333333336</v>
+      </c>
+      <c r="C519" s="3">
+        <v>45983.708333333336</v>
+      </c>
+    </row>
+    <row r="520" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A520" s="2">
+        <v>1</v>
+      </c>
+      <c r="B520" s="3">
+        <v>45984.333333333336</v>
+      </c>
+      <c r="C520" s="3">
+        <v>45984.708333333336</v>
+      </c>
+    </row>
+    <row r="521" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A521" s="2">
+        <v>1</v>
+      </c>
+      <c r="B521" s="3">
+        <v>45985.333333333336</v>
+      </c>
+      <c r="C521" s="3">
+        <v>45985.708333333336</v>
+      </c>
+    </row>
+    <row r="522" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A522" s="2">
+        <v>1</v>
+      </c>
+      <c r="B522" s="3">
+        <v>45986.333333333336</v>
+      </c>
+      <c r="C522" s="3">
+        <v>45986.708333333336</v>
+      </c>
+    </row>
+    <row r="523" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A523" s="2">
+        <v>1</v>
+      </c>
+      <c r="B523" s="3">
+        <v>45987.333333333336</v>
+      </c>
+      <c r="C523" s="3">
+        <v>45987.708333333336</v>
+      </c>
+    </row>
+    <row r="524" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A524" s="2">
+        <v>1</v>
+      </c>
+      <c r="B524" s="3">
+        <v>45988.333333333336</v>
+      </c>
+      <c r="C524" s="3">
+        <v>45988.708333333336</v>
+      </c>
+    </row>
+    <row r="525" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A525" s="2">
+        <v>1</v>
+      </c>
+      <c r="B525" s="3">
+        <v>45989.333333333336</v>
+      </c>
+      <c r="C525" s="3">
+        <v>45989.708333333336</v>
+      </c>
+    </row>
+    <row r="526" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A526" s="2">
+        <v>1</v>
+      </c>
+      <c r="B526" s="3">
+        <v>45990.333333333336</v>
+      </c>
+      <c r="C526" s="3">
+        <v>45990.708333333336</v>
+      </c>
+    </row>
+    <row r="527" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A527" s="2">
+        <v>1</v>
+      </c>
+      <c r="B527" s="3">
+        <v>45991.333333333336</v>
+      </c>
+      <c r="C527" s="3">
+        <v>45991.708333333336</v>
+      </c>
+    </row>
+    <row r="528" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A528" s="2">
+        <v>1</v>
+      </c>
+      <c r="B528" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C528" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="529" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A529" s="2">
+        <v>2</v>
+      </c>
+      <c r="B529" s="3">
+        <v>45962.333333333336</v>
+      </c>
+      <c r="C529" s="3">
+        <v>45962.708333333336</v>
+      </c>
+    </row>
+    <row r="530" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A530" s="2">
+        <v>2</v>
+      </c>
+      <c r="B530" s="3">
+        <v>45963.333333333336</v>
+      </c>
+      <c r="C530" s="3">
+        <v>45963.708333333336</v>
+      </c>
+    </row>
+    <row r="531" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A531" s="2">
+        <v>2</v>
+      </c>
+      <c r="B531" s="3">
+        <v>45964.333333333336</v>
+      </c>
+      <c r="C531" s="3">
+        <v>45964.708333333336</v>
+      </c>
+    </row>
+    <row r="532" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A532" s="2">
+        <v>2</v>
+      </c>
+      <c r="B532" s="3">
+        <v>45965.333333333336</v>
+      </c>
+      <c r="C532" s="3">
+        <v>45965.708333333336</v>
+      </c>
+    </row>
+    <row r="533" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A533" s="2">
+        <v>2</v>
+      </c>
+      <c r="B533" s="3">
+        <v>45966.333333333336</v>
+      </c>
+      <c r="C533" s="3">
+        <v>45966.708333333336</v>
+      </c>
+    </row>
+    <row r="534" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A534" s="2">
+        <v>2</v>
+      </c>
+      <c r="B534" s="3">
+        <v>45967.333333333336</v>
+      </c>
+      <c r="C534" s="3">
+        <v>45967.708333333336</v>
+      </c>
+    </row>
+    <row r="535" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A535" s="2">
+        <v>2</v>
+      </c>
+      <c r="B535" s="3">
+        <v>45968.333333333336</v>
+      </c>
+      <c r="C535" s="3">
+        <v>45968.708333333336</v>
+      </c>
+    </row>
+    <row r="536" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A536" s="2">
+        <v>2</v>
+      </c>
+      <c r="B536" s="3">
+        <v>45969.333333333336</v>
+      </c>
+      <c r="C536" s="3">
+        <v>45969.708333333336</v>
+      </c>
+    </row>
+    <row r="537" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A537" s="2">
+        <v>2</v>
+      </c>
+      <c r="B537" s="3">
+        <v>45970.333333333336</v>
+      </c>
+      <c r="C537" s="3">
+        <v>45970.708333333336</v>
+      </c>
+    </row>
+    <row r="538" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A538" s="2">
+        <v>2</v>
+      </c>
+      <c r="B538" s="3">
+        <v>45971.333333333336</v>
+      </c>
+      <c r="C538" s="3">
+        <v>45971.708333333336</v>
+      </c>
+    </row>
+    <row r="539" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A539" s="2">
+        <v>2</v>
+      </c>
+      <c r="B539" s="3">
+        <v>45972.333333333336</v>
+      </c>
+      <c r="C539" s="3">
+        <v>45972.708333333336</v>
+      </c>
+    </row>
+    <row r="540" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A540" s="2">
+        <v>2</v>
+      </c>
+      <c r="B540" s="3">
+        <v>45973.333333333336</v>
+      </c>
+      <c r="C540" s="3">
+        <v>45973.708333333336</v>
+      </c>
+    </row>
+    <row r="541" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A541" s="2">
+        <v>2</v>
+      </c>
+      <c r="B541" s="3">
+        <v>45974.333333333336</v>
+      </c>
+      <c r="C541" s="3">
+        <v>45974.708333333336</v>
+      </c>
+    </row>
+    <row r="542" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A542" s="2">
+        <v>2</v>
+      </c>
+      <c r="B542" s="3">
+        <v>45975.333333333336</v>
+      </c>
+      <c r="C542" s="3">
+        <v>45975.708333333336</v>
+      </c>
+    </row>
+    <row r="543" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A543" s="2">
+        <v>2</v>
+      </c>
+      <c r="B543" s="3">
+        <v>45976.333333333336</v>
+      </c>
+      <c r="C543" s="3">
+        <v>45976.708333333336</v>
+      </c>
+    </row>
+    <row r="544" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A544" s="2">
+        <v>2</v>
+      </c>
+      <c r="B544" s="3">
+        <v>45977.333333333336</v>
+      </c>
+      <c r="C544" s="3">
+        <v>45977.708333333336</v>
+      </c>
+    </row>
+    <row r="545" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A545" s="2">
+        <v>2</v>
+      </c>
+      <c r="B545" s="3">
+        <v>45978.333333333336</v>
+      </c>
+      <c r="C545" s="3">
+        <v>45978.708333333336</v>
+      </c>
+    </row>
+    <row r="546" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A546" s="2">
+        <v>2</v>
+      </c>
+      <c r="B546" s="3">
+        <v>45979.333333333336</v>
+      </c>
+      <c r="C546" s="3">
+        <v>45979.708333333336</v>
+      </c>
+    </row>
+    <row r="547" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A547" s="2">
+        <v>2</v>
+      </c>
+      <c r="B547" s="3">
+        <v>45980.333333333336</v>
+      </c>
+      <c r="C547" s="3">
+        <v>45980.708333333336</v>
+      </c>
+    </row>
+    <row r="548" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A548" s="2">
+        <v>2</v>
+      </c>
+      <c r="B548" s="3">
+        <v>45981.333333333336</v>
+      </c>
+      <c r="C548" s="3">
+        <v>45981.708333333336</v>
+      </c>
+    </row>
+    <row r="549" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A549" s="2">
+        <v>2</v>
+      </c>
+      <c r="B549" s="3">
+        <v>45982.333333333336</v>
+      </c>
+      <c r="C549" s="3">
+        <v>45982.708333333336</v>
+      </c>
+    </row>
+    <row r="550" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A550" s="2">
+        <v>2</v>
+      </c>
+      <c r="B550" s="3">
+        <v>45983.333333333336</v>
+      </c>
+      <c r="C550" s="3">
+        <v>45983.708333333336</v>
+      </c>
+    </row>
+    <row r="551" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A551" s="2">
+        <v>2</v>
+      </c>
+      <c r="B551" s="3">
+        <v>45984.333333333336</v>
+      </c>
+      <c r="C551" s="3">
+        <v>45984.708333333336</v>
+      </c>
+    </row>
+    <row r="552" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A552" s="2">
+        <v>2</v>
+      </c>
+      <c r="B552" s="3">
+        <v>45985.333333333336</v>
+      </c>
+      <c r="C552" s="3">
+        <v>45985.708333333336</v>
+      </c>
+    </row>
+    <row r="553" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A553" s="2">
+        <v>2</v>
+      </c>
+      <c r="B553" s="3">
+        <v>45986.333333333336</v>
+      </c>
+      <c r="C553" s="3">
+        <v>45986.708333333336</v>
+      </c>
+    </row>
+    <row r="554" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A554" s="2">
+        <v>2</v>
+      </c>
+      <c r="B554" s="3">
+        <v>45987.333333333336</v>
+      </c>
+      <c r="C554" s="3">
+        <v>45987.708333333336</v>
+      </c>
+    </row>
+    <row r="555" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A555" s="2">
+        <v>2</v>
+      </c>
+      <c r="B555" s="3">
+        <v>45988.333333333336</v>
+      </c>
+      <c r="C555" s="3">
+        <v>45988.708333333336</v>
+      </c>
+    </row>
+    <row r="556" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A556" s="2">
+        <v>2</v>
+      </c>
+      <c r="B556" s="3">
+        <v>45989.333333333336</v>
+      </c>
+      <c r="C556" s="3">
+        <v>45989.708333333336</v>
+      </c>
+    </row>
+    <row r="557" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A557" s="2">
+        <v>2</v>
+      </c>
+      <c r="B557" s="3">
+        <v>45990.333333333336</v>
+      </c>
+      <c r="C557" s="3">
+        <v>45990.708333333336</v>
+      </c>
+    </row>
+    <row r="558" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A558" s="2">
+        <v>2</v>
+      </c>
+      <c r="B558" s="3">
+        <v>45991.333333333336</v>
+      </c>
+      <c r="C558" s="3">
+        <v>45991.708333333336</v>
+      </c>
+    </row>
+    <row r="559" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A559" s="2">
+        <v>2</v>
+      </c>
+      <c r="B559" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C559" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="560" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A560" s="2">
+        <v>3</v>
+      </c>
+      <c r="B560" s="3">
+        <v>45962.333333333336</v>
+      </c>
+      <c r="C560" s="3">
+        <v>45962.708333333336</v>
+      </c>
+    </row>
+    <row r="561" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A561" s="2">
+        <v>3</v>
+      </c>
+      <c r="B561" s="3">
+        <v>45963.333333333336</v>
+      </c>
+      <c r="C561" s="3">
+        <v>45963.708333333336</v>
+      </c>
+    </row>
+    <row r="562" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A562" s="2">
+        <v>3</v>
+      </c>
+      <c r="B562" s="3">
+        <v>45964.333333333336</v>
+      </c>
+      <c r="C562" s="3">
+        <v>45964.708333333336</v>
+      </c>
+    </row>
+    <row r="563" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A563" s="2">
+        <v>3</v>
+      </c>
+      <c r="B563" s="3">
+        <v>45965.333333333336</v>
+      </c>
+      <c r="C563" s="3">
+        <v>45965.708333333336</v>
+      </c>
+    </row>
+    <row r="564" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A564" s="2">
+        <v>3</v>
+      </c>
+      <c r="B564" s="3">
+        <v>45966.333333333336</v>
+      </c>
+      <c r="C564" s="3">
+        <v>45966.708333333336</v>
+      </c>
+    </row>
+    <row r="565" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A565" s="2">
+        <v>3</v>
+      </c>
+      <c r="B565" s="3">
+        <v>45967.333333333336</v>
+      </c>
+      <c r="C565" s="3">
+        <v>45967.708333333336</v>
+      </c>
+    </row>
+    <row r="566" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A566" s="2">
+        <v>3</v>
+      </c>
+      <c r="B566" s="3">
+        <v>45968.333333333336</v>
+      </c>
+      <c r="C566" s="3">
+        <v>45968.708333333336</v>
+      </c>
+    </row>
+    <row r="567" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A567" s="2">
+        <v>3</v>
+      </c>
+      <c r="B567" s="3">
+        <v>45969.333333333336</v>
+      </c>
+      <c r="C567" s="3">
+        <v>45969.708333333336</v>
+      </c>
+    </row>
+    <row r="568" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A568" s="2">
+        <v>3</v>
+      </c>
+      <c r="B568" s="3">
+        <v>45970.333333333336</v>
+      </c>
+      <c r="C568" s="3">
+        <v>45970.708333333336</v>
+      </c>
+    </row>
+    <row r="569" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A569" s="2">
+        <v>3</v>
+      </c>
+      <c r="B569" s="3">
+        <v>45971.333333333336</v>
+      </c>
+      <c r="C569" s="3">
+        <v>45971.708333333336</v>
+      </c>
+    </row>
+    <row r="570" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A570" s="2">
+        <v>3</v>
+      </c>
+      <c r="B570" s="3">
+        <v>45972.333333333336</v>
+      </c>
+      <c r="C570" s="3">
+        <v>45972.708333333336</v>
+      </c>
+    </row>
+    <row r="571" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A571" s="2">
+        <v>3</v>
+      </c>
+      <c r="B571" s="3">
+        <v>45973.333333333336</v>
+      </c>
+      <c r="C571" s="3">
+        <v>45973.708333333336</v>
+      </c>
+    </row>
+    <row r="572" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A572" s="2">
+        <v>3</v>
+      </c>
+      <c r="B572" s="3">
+        <v>45974.333333333336</v>
+      </c>
+      <c r="C572" s="3">
+        <v>45974.708333333336</v>
+      </c>
+    </row>
+    <row r="573" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A573" s="2">
+        <v>3</v>
+      </c>
+      <c r="B573" s="3">
+        <v>45975.333333333336</v>
+      </c>
+      <c r="C573" s="3">
+        <v>45975.708333333336</v>
+      </c>
+    </row>
+    <row r="574" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A574" s="2">
+        <v>3</v>
+      </c>
+      <c r="B574" s="3">
+        <v>45976.333333333336</v>
+      </c>
+      <c r="C574" s="3">
+        <v>45976.708333333336</v>
+      </c>
+    </row>
+    <row r="575" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A575" s="2">
+        <v>3</v>
+      </c>
+      <c r="B575" s="3">
+        <v>45977.333333333336</v>
+      </c>
+      <c r="C575" s="3">
+        <v>45977.708333333336</v>
+      </c>
+    </row>
+    <row r="576" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A576" s="2">
+        <v>3</v>
+      </c>
+      <c r="B576" s="3">
+        <v>45978.333333333336</v>
+      </c>
+      <c r="C576" s="3">
+        <v>45978.708333333336</v>
+      </c>
+    </row>
+    <row r="577" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A577" s="2">
+        <v>3</v>
+      </c>
+      <c r="B577" s="3">
+        <v>45979.333333333336</v>
+      </c>
+      <c r="C577" s="3">
+        <v>45979.708333333336</v>
+      </c>
+    </row>
+    <row r="578" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A578" s="2">
+        <v>3</v>
+      </c>
+      <c r="B578" s="3">
+        <v>45980.333333333336</v>
+      </c>
+      <c r="C578" s="3">
+        <v>45980.708333333336</v>
+      </c>
+    </row>
+    <row r="579" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A579" s="2">
+        <v>3</v>
+      </c>
+      <c r="B579" s="3">
+        <v>45981.333333333336</v>
+      </c>
+      <c r="C579" s="3">
+        <v>45981.708333333336</v>
+      </c>
+    </row>
+    <row r="580" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A580" s="2">
+        <v>3</v>
+      </c>
+      <c r="B580" s="3">
+        <v>45982.333333333336</v>
+      </c>
+      <c r="C580" s="3">
+        <v>45982.708333333336</v>
+      </c>
+    </row>
+    <row r="581" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A581" s="2">
+        <v>3</v>
+      </c>
+      <c r="B581" s="3">
+        <v>45983.333333333336</v>
+      </c>
+      <c r="C581" s="3">
+        <v>45983.708333333336</v>
+      </c>
+    </row>
+    <row r="582" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A582" s="2">
+        <v>3</v>
+      </c>
+      <c r="B582" s="3">
+        <v>45984.333333333336</v>
+      </c>
+      <c r="C582" s="3">
+        <v>45984.708333333336</v>
+      </c>
+    </row>
+    <row r="583" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A583" s="2">
+        <v>3</v>
+      </c>
+      <c r="B583" s="3">
+        <v>45985.333333333336</v>
+      </c>
+      <c r="C583" s="3">
+        <v>45985.708333333336</v>
+      </c>
+    </row>
+    <row r="584" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A584" s="2">
+        <v>3</v>
+      </c>
+      <c r="B584" s="3">
+        <v>45986.333333333336</v>
+      </c>
+      <c r="C584" s="3">
+        <v>45986.708333333336</v>
+      </c>
+    </row>
+    <row r="585" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A585" s="2">
+        <v>3</v>
+      </c>
+      <c r="B585" s="3">
+        <v>45987.333333333336</v>
+      </c>
+      <c r="C585" s="3">
+        <v>45987.708333333336</v>
+      </c>
+    </row>
+    <row r="586" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A586" s="2">
+        <v>3</v>
+      </c>
+      <c r="B586" s="3">
+        <v>45988.333333333336</v>
+      </c>
+      <c r="C586" s="3">
+        <v>45988.708333333336</v>
+      </c>
+    </row>
+    <row r="587" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A587" s="2">
+        <v>3</v>
+      </c>
+      <c r="B587" s="3">
+        <v>45989.333333333336</v>
+      </c>
+      <c r="C587" s="3">
+        <v>45989.708333333336</v>
+      </c>
+    </row>
+    <row r="588" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A588" s="2">
+        <v>3</v>
+      </c>
+      <c r="B588" s="3">
+        <v>45990.333333333336</v>
+      </c>
+      <c r="C588" s="3">
+        <v>45990.708333333336</v>
+      </c>
+    </row>
+    <row r="589" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A589" s="2">
+        <v>3</v>
+      </c>
+      <c r="B589" s="3">
+        <v>45991.333333333336</v>
+      </c>
+      <c r="C589" s="3">
+        <v>45991.708333333336</v>
+      </c>
+    </row>
+    <row r="590" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A590" s="2">
+        <v>3</v>
+      </c>
+      <c r="B590" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C590" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="591" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A591" s="2">
+        <v>1</v>
+      </c>
+      <c r="B591" s="3">
+        <v>45931.333333333336</v>
+      </c>
+      <c r="C591" s="3">
+        <v>45931.708333333336</v>
+      </c>
+    </row>
+    <row r="592" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A592" s="2">
+        <v>1</v>
+      </c>
+      <c r="B592" s="3">
+        <v>45932.333333333336</v>
+      </c>
+      <c r="C592" s="3">
+        <v>45932.708333333336</v>
+      </c>
+    </row>
+    <row r="593" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A593" s="2">
+        <v>1</v>
+      </c>
+      <c r="B593" s="3">
+        <v>45933.333333333336</v>
+      </c>
+      <c r="C593" s="3">
+        <v>45933.708333333336</v>
+      </c>
+    </row>
+    <row r="594" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A594" s="2">
+        <v>1</v>
+      </c>
+      <c r="B594" s="3">
+        <v>45934.333333333336</v>
+      </c>
+      <c r="C594" s="3">
+        <v>45934.708333333336</v>
+      </c>
+    </row>
+    <row r="595" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A595" s="2">
+        <v>1</v>
+      </c>
+      <c r="B595" s="3">
+        <v>45935.333333333336</v>
+      </c>
+      <c r="C595" s="3">
+        <v>45935.708333333336</v>
+      </c>
+    </row>
+    <row r="596" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A596" s="2">
+        <v>1</v>
+      </c>
+      <c r="B596" s="3">
+        <v>45936.333333333336</v>
+      </c>
+      <c r="C596" s="3">
+        <v>45936.708333333336</v>
+      </c>
+    </row>
+    <row r="597" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A597" s="2">
+        <v>1</v>
+      </c>
+      <c r="B597" s="3">
+        <v>45937.333333333336</v>
+      </c>
+      <c r="C597" s="3">
+        <v>45937.708333333336</v>
+      </c>
+    </row>
+    <row r="598" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A598" s="2">
+        <v>1</v>
+      </c>
+      <c r="B598" s="3">
+        <v>45938.333333333336</v>
+      </c>
+      <c r="C598" s="3">
+        <v>45938.708333333336</v>
+      </c>
+    </row>
+    <row r="599" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A599" s="2">
+        <v>1</v>
+      </c>
+      <c r="B599" s="3">
+        <v>45939.333333333336</v>
+      </c>
+      <c r="C599" s="3">
+        <v>45939.708333333336</v>
+      </c>
+    </row>
+    <row r="600" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A600" s="2">
+        <v>1</v>
+      </c>
+      <c r="B600" s="3">
+        <v>45940.333333333336</v>
+      </c>
+      <c r="C600" s="3">
+        <v>45940.708333333336</v>
+      </c>
+    </row>
+    <row r="601" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A601" s="2">
+        <v>1</v>
+      </c>
+      <c r="B601" s="3">
+        <v>45941.333333333336</v>
+      </c>
+      <c r="C601" s="3">
+        <v>45941.708333333336</v>
+      </c>
+    </row>
+    <row r="602" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A602" s="2">
+        <v>1</v>
+      </c>
+      <c r="B602" s="3">
+        <v>45942.333333333336</v>
+      </c>
+      <c r="C602" s="3">
+        <v>45942.708333333336</v>
+      </c>
+    </row>
+    <row r="603" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A603" s="2">
+        <v>1</v>
+      </c>
+      <c r="B603" s="3">
+        <v>45943.333333333336</v>
+      </c>
+      <c r="C603" s="3">
+        <v>45943.708333333336</v>
+      </c>
+    </row>
+    <row r="604" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A604" s="2">
+        <v>1</v>
+      </c>
+      <c r="B604" s="3">
+        <v>45944.333333333336</v>
+      </c>
+      <c r="C604" s="3">
+        <v>45944.708333333336</v>
+      </c>
+    </row>
+    <row r="605" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A605" s="2">
+        <v>1</v>
+      </c>
+      <c r="B605" s="3">
+        <v>45945.333333333336</v>
+      </c>
+      <c r="C605" s="3">
+        <v>45945.708333333336</v>
+      </c>
+    </row>
+    <row r="606" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A606" s="2">
+        <v>1</v>
+      </c>
+      <c r="B606" s="3">
+        <v>45946.333333333336</v>
+      </c>
+      <c r="C606" s="3">
+        <v>45946.708333333336</v>
+      </c>
+    </row>
+    <row r="607" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A607" s="2">
+        <v>1</v>
+      </c>
+      <c r="B607" s="3">
+        <v>45947.333333333336</v>
+      </c>
+      <c r="C607" s="3">
+        <v>45947.708333333336</v>
+      </c>
+    </row>
+    <row r="608" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A608" s="2">
+        <v>1</v>
+      </c>
+      <c r="B608" s="3">
+        <v>45948.333333333336</v>
+      </c>
+      <c r="C608" s="3">
+        <v>45948.708333333336</v>
+      </c>
+    </row>
+    <row r="609" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A609" s="2">
+        <v>1</v>
+      </c>
+      <c r="B609" s="3">
+        <v>45949.333333333336</v>
+      </c>
+      <c r="C609" s="3">
+        <v>45949.708333333336</v>
+      </c>
+    </row>
+    <row r="610" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A610" s="2">
+        <v>1</v>
+      </c>
+      <c r="B610" s="3">
+        <v>45950.333333333336</v>
+      </c>
+      <c r="C610" s="3">
+        <v>45950.708333333336</v>
+      </c>
+    </row>
+    <row r="611" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A611" s="2">
+        <v>1</v>
+      </c>
+      <c r="B611" s="3">
+        <v>45951.333333333336</v>
+      </c>
+      <c r="C611" s="3">
+        <v>45951.708333333336</v>
+      </c>
+    </row>
+    <row r="612" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A612" s="2">
+        <v>1</v>
+      </c>
+      <c r="B612" s="3">
+        <v>45952.333333333336</v>
+      </c>
+      <c r="C612" s="3">
+        <v>45952.708333333336</v>
+      </c>
+    </row>
+    <row r="613" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A613" s="2">
+        <v>1</v>
+      </c>
+      <c r="B613" s="3">
+        <v>45953.333333333336</v>
+      </c>
+      <c r="C613" s="3">
+        <v>45953.708333333336</v>
+      </c>
+    </row>
+    <row r="614" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A614" s="2">
+        <v>1</v>
+      </c>
+      <c r="B614" s="3">
+        <v>45954.333333333336</v>
+      </c>
+      <c r="C614" s="3">
+        <v>45954.708333333336</v>
+      </c>
+    </row>
+    <row r="615" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A615" s="2">
+        <v>1</v>
+      </c>
+      <c r="B615" s="3">
+        <v>45955.333333333336</v>
+      </c>
+      <c r="C615" s="3">
+        <v>45955.708333333336</v>
+      </c>
+    </row>
+    <row r="616" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A616" s="2">
+        <v>1</v>
+      </c>
+      <c r="B616" s="3">
+        <v>45956.333333333336</v>
+      </c>
+      <c r="C616" s="3">
+        <v>45956.708333333336</v>
+      </c>
+    </row>
+    <row r="617" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A617" s="2">
+        <v>1</v>
+      </c>
+      <c r="B617" s="3">
+        <v>45957.333333333336</v>
+      </c>
+      <c r="C617" s="3">
+        <v>45957.708333333336</v>
+      </c>
+    </row>
+    <row r="618" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A618" s="2">
+        <v>1</v>
+      </c>
+      <c r="B618" s="3">
+        <v>45958.333333333336</v>
+      </c>
+      <c r="C618" s="3">
+        <v>45958.708333333336</v>
+      </c>
+    </row>
+    <row r="619" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A619" s="2">
+        <v>1</v>
+      </c>
+      <c r="B619" s="3">
+        <v>45959.333333333336</v>
+      </c>
+      <c r="C619" s="3">
+        <v>45959.708333333336</v>
+      </c>
+    </row>
+    <row r="620" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A620" s="2">
+        <v>1</v>
+      </c>
+      <c r="B620" s="3">
+        <v>45960.333333333336</v>
+      </c>
+      <c r="C620" s="3">
+        <v>45960.708333333336</v>
+      </c>
+    </row>
+    <row r="621" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A621" s="2">
+        <v>1</v>
+      </c>
+      <c r="B621" s="3">
+        <v>45961.333333333336</v>
+      </c>
+      <c r="C621" s="3">
+        <v>45961.708333333336</v>
+      </c>
+    </row>
+    <row r="622" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A622" s="2">
+        <v>2</v>
+      </c>
+      <c r="B622" s="3">
+        <v>45931.333333333336</v>
+      </c>
+      <c r="C622" s="3">
+        <v>45931.708333333336</v>
+      </c>
+    </row>
+    <row r="623" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A623" s="2">
+        <v>2</v>
+      </c>
+      <c r="B623" s="3">
+        <v>45932.333333333336</v>
+      </c>
+      <c r="C623" s="3">
+        <v>45932.708333333336</v>
+      </c>
+    </row>
+    <row r="624" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A624" s="2">
+        <v>2</v>
+      </c>
+      <c r="B624" s="3">
+        <v>45933.333333333336</v>
+      </c>
+      <c r="C624" s="3">
+        <v>45933.708333333336</v>
+      </c>
+    </row>
+    <row r="625" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A625" s="2">
+        <v>2</v>
+      </c>
+      <c r="B625" s="3">
+        <v>45934.333333333336</v>
+      </c>
+      <c r="C625" s="3">
+        <v>45934.708333333336</v>
+      </c>
+    </row>
+    <row r="626" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A626" s="2">
+        <v>2</v>
+      </c>
+      <c r="B626" s="3">
+        <v>45935.333333333336</v>
+      </c>
+      <c r="C626" s="3">
+        <v>45935.708333333336</v>
+      </c>
+    </row>
+    <row r="627" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A627" s="2">
+        <v>2</v>
+      </c>
+      <c r="B627" s="3">
+        <v>45936.333333333336</v>
+      </c>
+      <c r="C627" s="3">
+        <v>45936.708333333336</v>
+      </c>
+    </row>
+    <row r="628" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A628" s="2">
+        <v>2</v>
+      </c>
+      <c r="B628" s="3">
+        <v>45937.333333333336</v>
+      </c>
+      <c r="C628" s="3">
+        <v>45937.708333333336</v>
+      </c>
+    </row>
+    <row r="629" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A629" s="2">
+        <v>2</v>
+      </c>
+      <c r="B629" s="3">
+        <v>45938.333333333336</v>
+      </c>
+      <c r="C629" s="3">
+        <v>45938.708333333336</v>
+      </c>
+    </row>
+    <row r="630" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A630" s="2">
+        <v>2</v>
+      </c>
+      <c r="B630" s="3">
+        <v>45939.333333333336</v>
+      </c>
+      <c r="C630" s="3">
+        <v>45939.708333333336</v>
+      </c>
+    </row>
+    <row r="631" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A631" s="2">
+        <v>2</v>
+      </c>
+      <c r="B631" s="3">
+        <v>45940.333333333336</v>
+      </c>
+      <c r="C631" s="3">
+        <v>45940.708333333336</v>
+      </c>
+    </row>
+    <row r="632" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A632" s="2">
+        <v>2</v>
+      </c>
+      <c r="B632" s="3">
+        <v>45941.333333333336</v>
+      </c>
+      <c r="C632" s="3">
+        <v>45941.708333333336</v>
+      </c>
+    </row>
+    <row r="633" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A633" s="2">
+        <v>2</v>
+      </c>
+      <c r="B633" s="3">
+        <v>45942.333333333336</v>
+      </c>
+      <c r="C633" s="3">
+        <v>45942.708333333336</v>
+      </c>
+    </row>
+    <row r="634" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A634" s="2">
+        <v>2</v>
+      </c>
+      <c r="B634" s="3">
+        <v>45943.333333333336</v>
+      </c>
+      <c r="C634" s="3">
+        <v>45943.708333333336</v>
+      </c>
+    </row>
+    <row r="635" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A635" s="2">
+        <v>2</v>
+      </c>
+      <c r="B635" s="3">
+        <v>45944.333333333336</v>
+      </c>
+      <c r="C635" s="3">
+        <v>45944.708333333336</v>
+      </c>
+    </row>
+    <row r="636" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A636" s="2">
+        <v>2</v>
+      </c>
+      <c r="B636" s="3">
+        <v>45945.333333333336</v>
+      </c>
+      <c r="C636" s="3">
+        <v>45945.708333333336</v>
+      </c>
+    </row>
+    <row r="637" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A637" s="2">
+        <v>2</v>
+      </c>
+      <c r="B637" s="3">
+        <v>45946.333333333336</v>
+      </c>
+      <c r="C637" s="3">
+        <v>45946.708333333336</v>
+      </c>
+    </row>
+    <row r="638" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A638" s="2">
+        <v>2</v>
+      </c>
+      <c r="B638" s="3">
+        <v>45947.333333333336</v>
+      </c>
+      <c r="C638" s="3">
+        <v>45947.708333333336</v>
+      </c>
+    </row>
+    <row r="639" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A639" s="2">
+        <v>2</v>
+      </c>
+      <c r="B639" s="3">
+        <v>45948.333333333336</v>
+      </c>
+      <c r="C639" s="3">
+        <v>45948.708333333336</v>
+      </c>
+    </row>
+    <row r="640" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A640" s="2">
+        <v>2</v>
+      </c>
+      <c r="B640" s="3">
+        <v>45949.333333333336</v>
+      </c>
+      <c r="C640" s="3">
+        <v>45949.708333333336</v>
+      </c>
+    </row>
+    <row r="641" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A641" s="2">
+        <v>2</v>
+      </c>
+      <c r="B641" s="3">
+        <v>45950.333333333336</v>
+      </c>
+      <c r="C641" s="3">
+        <v>45950.708333333336</v>
+      </c>
+    </row>
+    <row r="642" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A642" s="2">
+        <v>2</v>
+      </c>
+      <c r="B642" s="3">
+        <v>45951.333333333336</v>
+      </c>
+      <c r="C642" s="3">
+        <v>45951.708333333336</v>
+      </c>
+    </row>
+    <row r="643" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A643" s="2">
+        <v>2</v>
+      </c>
+      <c r="B643" s="3">
+        <v>45952.333333333336</v>
+      </c>
+      <c r="C643" s="3">
+        <v>45952.708333333336</v>
+      </c>
+    </row>
+    <row r="644" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A644" s="2">
+        <v>2</v>
+      </c>
+      <c r="B644" s="3">
+        <v>45953.333333333336</v>
+      </c>
+      <c r="C644" s="3">
+        <v>45953.708333333336</v>
+      </c>
+    </row>
+    <row r="645" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A645" s="2">
+        <v>2</v>
+      </c>
+      <c r="B645" s="3">
+        <v>45954.333333333336</v>
+      </c>
+      <c r="C645" s="3">
+        <v>45954.708333333336</v>
+      </c>
+    </row>
+    <row r="646" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A646" s="2">
+        <v>2</v>
+      </c>
+      <c r="B646" s="3">
+        <v>45955.333333333336</v>
+      </c>
+      <c r="C646" s="3">
+        <v>45955.708333333336</v>
+      </c>
+    </row>
+    <row r="647" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A647" s="2">
+        <v>2</v>
+      </c>
+      <c r="B647" s="3">
+        <v>45956.333333333336</v>
+      </c>
+      <c r="C647" s="3">
+        <v>45956.708333333336</v>
+      </c>
+    </row>
+    <row r="648" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A648" s="2">
+        <v>2</v>
+      </c>
+      <c r="B648" s="3">
+        <v>45957.333333333336</v>
+      </c>
+      <c r="C648" s="3">
+        <v>45957.708333333336</v>
+      </c>
+    </row>
+    <row r="649" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A649" s="2">
+        <v>2</v>
+      </c>
+      <c r="B649" s="3">
+        <v>45958.333333333336</v>
+      </c>
+      <c r="C649" s="3">
+        <v>45958.708333333336</v>
+      </c>
+    </row>
+    <row r="650" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A650" s="2">
+        <v>2</v>
+      </c>
+      <c r="B650" s="3">
+        <v>45959.333333333336</v>
+      </c>
+      <c r="C650" s="3">
+        <v>45959.708333333336</v>
+      </c>
+    </row>
+    <row r="651" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A651" s="2">
+        <v>2</v>
+      </c>
+      <c r="B651" s="3">
+        <v>45960.333333333336</v>
+      </c>
+      <c r="C651" s="3">
+        <v>45960.708333333336</v>
+      </c>
+    </row>
+    <row r="652" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A652" s="2">
+        <v>2</v>
+      </c>
+      <c r="B652" s="3">
+        <v>45961.333333333336</v>
+      </c>
+      <c r="C652" s="3">
+        <v>45961.708333333336</v>
+      </c>
+    </row>
+    <row r="653" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A653" s="2">
+        <v>3</v>
+      </c>
+      <c r="B653" s="3">
+        <v>45931.333333333336</v>
+      </c>
+      <c r="C653" s="3">
+        <v>45931.708333333336</v>
+      </c>
+    </row>
+    <row r="654" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A654" s="2">
+        <v>3</v>
+      </c>
+      <c r="B654" s="3">
+        <v>45932.333333333336</v>
+      </c>
+      <c r="C654" s="3">
+        <v>45932.708333333336</v>
+      </c>
+    </row>
+    <row r="655" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A655" s="2">
+        <v>3</v>
+      </c>
+      <c r="B655" s="3">
+        <v>45933.333333333336</v>
+      </c>
+      <c r="C655" s="3">
+        <v>45933.708333333336</v>
+      </c>
+    </row>
+    <row r="656" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A656" s="2">
+        <v>3</v>
+      </c>
+      <c r="B656" s="3">
+        <v>45934.333333333336</v>
+      </c>
+      <c r="C656" s="3">
+        <v>45934.708333333336</v>
+      </c>
+    </row>
+    <row r="657" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A657" s="2">
+        <v>3</v>
+      </c>
+      <c r="B657" s="3">
+        <v>45935.333333333336</v>
+      </c>
+      <c r="C657" s="3">
+        <v>45935.708333333336</v>
+      </c>
+    </row>
+    <row r="658" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A658" s="2">
+        <v>3</v>
+      </c>
+      <c r="B658" s="3">
+        <v>45936.333333333336</v>
+      </c>
+      <c r="C658" s="3">
+        <v>45936.708333333336</v>
+      </c>
+    </row>
+    <row r="659" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A659" s="2">
+        <v>3</v>
+      </c>
+      <c r="B659" s="3">
+        <v>45937.333333333336</v>
+      </c>
+      <c r="C659" s="3">
+        <v>45937.708333333336</v>
+      </c>
+    </row>
+    <row r="660" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A660" s="2">
+        <v>3</v>
+      </c>
+      <c r="B660" s="3">
+        <v>45938.333333333336</v>
+      </c>
+      <c r="C660" s="3">
+        <v>45938.708333333336</v>
+      </c>
+    </row>
+    <row r="661" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A661" s="2">
+        <v>3</v>
+      </c>
+      <c r="B661" s="3">
+        <v>45939.333333333336</v>
+      </c>
+      <c r="C661" s="3">
+        <v>45939.708333333336</v>
+      </c>
+    </row>
+    <row r="662" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A662" s="2">
+        <v>3</v>
+      </c>
+      <c r="B662" s="3">
+        <v>45940.333333333336</v>
+      </c>
+      <c r="C662" s="3">
+        <v>45940.708333333336</v>
+      </c>
+    </row>
+    <row r="663" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A663" s="2">
+        <v>3</v>
+      </c>
+      <c r="B663" s="3">
+        <v>45941.333333333336</v>
+      </c>
+      <c r="C663" s="3">
+        <v>45941.708333333336</v>
+      </c>
+    </row>
+    <row r="664" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A664" s="2">
+        <v>3</v>
+      </c>
+      <c r="B664" s="3">
+        <v>45942.333333333336</v>
+      </c>
+      <c r="C664" s="3">
+        <v>45942.708333333336</v>
+      </c>
+    </row>
+    <row r="665" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A665" s="2">
+        <v>3</v>
+      </c>
+      <c r="B665" s="3">
+        <v>45943.333333333336</v>
+      </c>
+      <c r="C665" s="3">
+        <v>45943.708333333336</v>
+      </c>
+    </row>
+    <row r="666" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A666" s="2">
+        <v>3</v>
+      </c>
+      <c r="B666" s="3">
+        <v>45944.333333333336</v>
+      </c>
+      <c r="C666" s="3">
+        <v>45944.708333333336</v>
+      </c>
+    </row>
+    <row r="667" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A667" s="2">
+        <v>3</v>
+      </c>
+      <c r="B667" s="3">
+        <v>45945.333333333336</v>
+      </c>
+      <c r="C667" s="3">
+        <v>45945.708333333336</v>
+      </c>
+    </row>
+    <row r="668" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A668" s="2">
+        <v>3</v>
+      </c>
+      <c r="B668" s="3">
+        <v>45946.333333333336</v>
+      </c>
+      <c r="C668" s="3">
+        <v>45946.708333333336</v>
+      </c>
+    </row>
+    <row r="669" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A669" s="2">
+        <v>3</v>
+      </c>
+      <c r="B669" s="3">
+        <v>45947.333333333336</v>
+      </c>
+      <c r="C669" s="3">
+        <v>45947.708333333336</v>
+      </c>
+    </row>
+    <row r="670" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A670" s="2">
+        <v>3</v>
+      </c>
+      <c r="B670" s="3">
+        <v>45948.333333333336</v>
+      </c>
+      <c r="C670" s="3">
+        <v>45948.708333333336</v>
+      </c>
+    </row>
+    <row r="671" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A671" s="2">
+        <v>3</v>
+      </c>
+      <c r="B671" s="3">
+        <v>45949.333333333336</v>
+      </c>
+      <c r="C671" s="3">
+        <v>45949.708333333336</v>
+      </c>
+    </row>
+    <row r="672" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A672" s="2">
+        <v>3</v>
+      </c>
+      <c r="B672" s="3">
+        <v>45950.333333333336</v>
+      </c>
+      <c r="C672" s="3">
+        <v>45950.708333333336</v>
+      </c>
+    </row>
+    <row r="673" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A673" s="2">
+        <v>3</v>
+      </c>
+      <c r="B673" s="3">
+        <v>45951.333333333336</v>
+      </c>
+      <c r="C673" s="3">
+        <v>45951.708333333336</v>
+      </c>
+    </row>
+    <row r="674" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A674" s="2">
+        <v>3</v>
+      </c>
+      <c r="B674" s="3">
+        <v>45952.333333333336</v>
+      </c>
+      <c r="C674" s="3">
+        <v>45952.708333333336</v>
+      </c>
+    </row>
+    <row r="675" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A675" s="2">
+        <v>3</v>
+      </c>
+      <c r="B675" s="3">
+        <v>45953.333333333336</v>
+      </c>
+      <c r="C675" s="3">
+        <v>45953.708333333336</v>
+      </c>
+    </row>
+    <row r="676" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A676" s="2">
+        <v>3</v>
+      </c>
+      <c r="B676" s="3">
+        <v>45954.333333333336</v>
+      </c>
+      <c r="C676" s="3">
+        <v>45954.708333333336</v>
+      </c>
+    </row>
+    <row r="677" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A677" s="2">
+        <v>3</v>
+      </c>
+      <c r="B677" s="3">
+        <v>45955.333333333336</v>
+      </c>
+      <c r="C677" s="3">
+        <v>45955.708333333336</v>
+      </c>
+    </row>
+    <row r="678" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A678" s="2">
+        <v>3</v>
+      </c>
+      <c r="B678" s="3">
+        <v>45956.333333333336</v>
+      </c>
+      <c r="C678" s="3">
+        <v>45956.708333333336</v>
+      </c>
+    </row>
+    <row r="679" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A679" s="2">
+        <v>3</v>
+      </c>
+      <c r="B679" s="3">
+        <v>45957.333333333336</v>
+      </c>
+      <c r="C679" s="3">
+        <v>45957.708333333336</v>
+      </c>
+    </row>
+    <row r="680" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A680" s="2">
+        <v>3</v>
+      </c>
+      <c r="B680" s="3">
+        <v>45958.333333333336</v>
+      </c>
+      <c r="C680" s="3">
+        <v>45958.708333333336</v>
+      </c>
+    </row>
+    <row r="681" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A681" s="2">
+        <v>3</v>
+      </c>
+      <c r="B681" s="3">
+        <v>45959.333333333336</v>
+      </c>
+      <c r="C681" s="3">
+        <v>45959.708333333336</v>
+      </c>
+    </row>
+    <row r="682" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A682" s="2">
+        <v>3</v>
+      </c>
+      <c r="B682" s="3">
+        <v>45960.333333333336</v>
+      </c>
+      <c r="C682" s="3">
+        <v>45960.708333333336</v>
+      </c>
+    </row>
+    <row r="683" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A683" s="2">
+        <v>3</v>
+      </c>
+      <c r="B683" s="3">
+        <v>45961.333333333336</v>
+      </c>
+      <c r="C683" s="3">
+        <v>45961.708333333336</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>